<commit_message>
Rebuild the syllabus on the chapter order of Database System Concepts (7th ed.)
- 60 sessions citing DSC sections and pages; 9 labs; guided self-study for
  abstract, hard-to-experiment topics (relational calculus, statistics
  estimation, most of recovery)
- Update grading scopes, materials, and constructivist questions
- Align the reading plan (computed session load) and the council brief
- Record the new structure in the project context

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/docs/IDB201_DSC_Reading_Plan.xlsx
+++ b/docs/IDB201_DSC_Reading_Plan.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -75,11 +75,6 @@
         <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -135,9 +130,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -568,13 +560,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>427</v>
+        <v>410</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.3289676425269646</v>
+        <v>0.3158705701078582</v>
       </c>
     </row>
     <row r="6">
@@ -589,13 +581,13 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.1987673343605547</v>
+        <v>0.211864406779661</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +796,7 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>Ch. 1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="G2" s="12" t="inlineStr">
@@ -847,12 +839,12 @@
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>Ch. 3, 4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>9–10, 14–17</t>
+          <t>4–8</t>
         </is>
       </c>
       <c r="H3" s="12" t="n">
@@ -890,12 +882,12 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>Ch. 5, 6, 7</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>20, 25–31, 34</t>
+          <t>9–14</t>
         </is>
       </c>
       <c r="H4" s="12" t="n">
@@ -933,12 +925,12 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Ch. 5, 6, 7</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>21–22, 27, 35</t>
+          <t>15–19</t>
         </is>
       </c>
       <c r="H5" s="12" t="n">
@@ -976,12 +968,12 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Ch. 6, 7, App. A</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>31, 33, 36</t>
+          <t>17–18</t>
         </is>
       </c>
       <c r="H6" s="12" t="n">
@@ -1019,12 +1011,12 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Ch. 2, 3</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>4–13</t>
+          <t>21–25</t>
         </is>
       </c>
       <c r="H7" s="12" t="n">
@@ -1062,12 +1054,12 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Ch. 8</t>
+          <t>C6</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>39–45</t>
+          <t>26–32</t>
         </is>
       </c>
       <c r="H8" s="12" t="n">
@@ -1269,12 +1261,12 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>35</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr"/>
@@ -1310,12 +1302,12 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>35–36</t>
         </is>
       </c>
       <c r="H14" s="12" t="n">
@@ -1353,12 +1345,12 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>36–40</t>
         </is>
       </c>
       <c r="H15" s="12" t="n">
@@ -1396,12 +1388,12 @@
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>41–43, 46</t>
         </is>
       </c>
       <c r="H16" s="12" t="n">
@@ -1439,16 +1431,16 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>44–46</t>
         </is>
       </c>
       <c r="H17" s="12" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
@@ -1482,12 +1474,12 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Ch. 10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>52–53</t>
+          <t>47–49, 53</t>
         </is>
       </c>
       <c r="H18" s="12" t="n">
@@ -1525,12 +1517,12 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Ch. 10</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>54–55</t>
+          <t>50–53</t>
         </is>
       </c>
       <c r="H19" s="12" t="n">
@@ -1561,27 +1553,27 @@
           <t>907–960</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Ch. 10</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>54</t>
         </is>
       </c>
       <c r="H20" s="12" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>Overview only: logging and the recovery algorithm (CLO7).</t>
+          <t>Abstract and hard to reproduce in a lab: one overview session (54), the rest is guided self-study (CLO7).</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1767,7 @@
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Ch. 9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -1934,25 +1926,25 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Ch. 4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6, 8</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr"/>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>Relational calculus and Codd's theorem are part of the academic orientation (CLO3).</t>
+          <t>Relational calculus is abstract and hard to experiment with, so it is guided self-study with a worksheet (CLO3).</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1974,7 @@
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Ch. 8</t>
+          <t>C6</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -2883,7 +2875,7 @@
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>Sessions 14–16</t>
+          <t>Sessions 5–6</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3571,7 @@
       </c>
       <c r="J34" s="12" t="inlineStr">
         <is>
-          <t>Taught with indexing (Ch. 9 of the course)</t>
+          <t>Session 17</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3699,7 @@
       </c>
       <c r="J37" s="12" t="inlineStr">
         <is>
-          <t>Python section only (session 36); JDBC/ODBC self-study</t>
+          <t>Python section (session 18); JDBC/ODBC self-study</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3831,7 @@
       </c>
       <c r="J40" s="12" t="inlineStr">
         <is>
-          <t>Transitive closure and expressive power (sessions 17, 33)</t>
+          <t>Transitive closure and expressive power (session 17)</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4199,7 @@
       </c>
       <c r="J49" s="12" t="inlineStr">
         <is>
-          <t>Sessions 11–12</t>
+          <t>Session 23</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4659,7 @@
       </c>
       <c r="J60" s="12" t="inlineStr">
         <is>
-          <t>MVDs and 4NF, brief (session 44)</t>
+          <t>MVDs and 4NF, overview (session 31)</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5399,7 @@
       </c>
       <c r="J78" s="12" t="inlineStr">
         <is>
-          <t>SQL injection (session 36); basis for DPY391</t>
+          <t>SQL injection (session 18); basis for DPY391</t>
         </is>
       </c>
     </row>
@@ -6843,7 +6835,7 @@
       </c>
       <c r="J113" s="12" t="inlineStr">
         <is>
-          <t>Composite indexes (Lab 8)</t>
+          <t>Composite indexes (Lab 7)</t>
         </is>
       </c>
     </row>
@@ -7535,19 +7527,19 @@
       <c r="G130" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="H130" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I130" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H130" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr">
+        <is>
+          <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J130" s="12" t="inlineStr">
         <is>
-          <t>Main ideas only</t>
+          <t>Abstract; guided self-study</t>
         </is>
       </c>
     </row>
@@ -8691,14 +8683,14 @@
       <c r="G158" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H158" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I158" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H158" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
+        </is>
+      </c>
+      <c r="I158" s="14" t="inlineStr">
+        <is>
+          <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J158" s="12" t="inlineStr"/>
@@ -8743,7 +8735,7 @@
       </c>
       <c r="J159" s="12" t="inlineStr">
         <is>
-          <t>Write-ahead logging</t>
+          <t>Write-ahead logging (overview, session 54)</t>
         </is>
       </c>
     </row>
@@ -8775,19 +8767,19 @@
       <c r="G160" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H160" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I160" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H160" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
+        </is>
+      </c>
+      <c r="I160" s="14" t="inlineStr">
+        <is>
+          <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J160" s="12" t="inlineStr">
         <is>
-          <t>Main ideas</t>
+          <t>Main ideas introduced in session 54; details self-study</t>
         </is>
       </c>
     </row>
@@ -9727,19 +9719,19 @@
       <c r="E183" s="12" t="n"/>
       <c r="F183" s="12" t="n"/>
       <c r="G183" s="12" t="n"/>
-      <c r="H183" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I183" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H183" s="14" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
+        </is>
+      </c>
+      <c r="I183" s="14" t="inlineStr">
+        <is>
+          <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
         <is>
-          <t>Session 17; the rest of the chapter is self-study</t>
+          <t>Guided self-study with a worksheet; reviewed in session 8</t>
         </is>
       </c>
     </row>
@@ -9925,16 +9917,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9945,7 +9936,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>DSC in-class sections</t>
+          <t>DSC chapters</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -9955,7 +9946,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Theory sessions (current syllabus)</t>
+          <t>Theory sessions</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -9965,24 +9956,19 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Recommendation</t>
+          <t>Verdict</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>1. Introduction</t>
+          <t>C1 Introduction</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>1.1–1.7</t>
+          <t>Ch. 1</t>
         </is>
       </c>
       <c r="C2" s="12" t="n">
@@ -9990,206 +9976,274 @@
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>1, 2, 3 (3)</t>
+          <t>1–2 (2)</t>
         </is>
       </c>
       <c r="E2" s="12" t="n">
-        <v>7.7</v>
+        <v>11.5</v>
       </c>
       <c r="F2" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>2–3. ER model and mapping</t>
+          <t>C2 Relational model and algebra</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>2.1–2.4, 6.1–6.7, 6.9</t>
+          <t>Ch. 2</t>
         </is>
       </c>
       <c r="C3" s="12" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>4–7, 9–12 (8)</t>
+          <t>4–6 (3)</t>
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>4. Relational algebra and calculus</t>
+          <t>C3 Introduction to SQL</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>2.5–2.6, online Ch. 27 (calculus)</t>
+          <t>Ch. 3</t>
         </is>
       </c>
       <c r="C4" s="12" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>14–17 (4)</t>
+          <t>9–12 (4)</t>
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>2.8</v>
+        <v>12.2</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Light in pages but heavy in proofs; online Ch. 27 adds reading.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>5–7. SQL</t>
+          <t>C4 Intermediate and advanced SQL</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>3.1–3.9, 4.1–4.6, 5.1 (Python), 5.4</t>
+          <t>Ch. 4, Ch. 5</t>
         </is>
       </c>
       <c r="C5" s="12" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>20–22, 25–27, 29–31, 34–36 (12)</t>
+          <t>15–18 (4)</t>
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>SQL syntax is also practised in 5 labs. Move session 31 (CTEs, window functions) to self-study (DSC 5.5).</t>
+        <v>15.2</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>8. Normalization</t>
+          <t>C5 E-R model</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>7.1–7.6, 7.8</t>
+          <t>Ch. 6</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>39–44 (6)</t>
+          <t>21–24 (4)</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>9. Storage, indexing, query processing</t>
+          <t>C6 Relational database design</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>13.1–13.3, 13.5, 14.1–14.3, 14.5–14.7, 15.1–15.5, 16.1–16.4</t>
+          <t>Ch. 7</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>121</v>
+        <v>39</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>47–50 (4)</t>
+          <t>26–31 (6)</t>
         </is>
       </c>
       <c r="E7" s="12" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>Too heavy</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Give this chapter 6 theory sessions (about 20 pages each): take session 31 and merge sessions 32–33 (Lab 5B) into one.</t>
+        <v>6.5</v>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>10. Transactions and recovery</t>
+          <t>C7 Storage and indexing</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>17.1–17.10, 18.1–18.2, 18.4, 18.8, 19.1–19.4</t>
+          <t>Ch. 12, Ch. 13, Ch. 14</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>52–55 (4)</t>
+          <t>35–38 (4)</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>Heavy but acceptable</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Keep; 19.x is taught as an overview only.</t>
+        <v>14</v>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>C8 Query processing and optimization</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Ch. 15, Ch. 16</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>56</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>41–45 (5)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>C9 Transactions and concurrency</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Ch. 17, Ch. 18</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>47–52 (6)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>C10 Recovery (mainly self-study)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Ch. 19</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>54 (1)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>In-class pages are read before class; each theory session is 45 minutes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise syllabus: 5 labs, one group project, no practical exam, final exam 50%
Merge the user's own edits of the uploaded workbook into the generator, then
apply the requested changes: reduce labs from 9 to 5 (SQL only), merge the two
assignments into one group project, remove the practical exam, set the final
exam to 50% (labs and CQ 10, PT1 5, PT2 5, project 30), move bag semantics and
Python to self-study. Update the council brief, reading plan and project notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GiH4cdiSXw8p9kG1C7Ltx9
</commit_message>
<xml_diff>
--- a/docs/IDB201_DSC_Reading_Plan.xlsx
+++ b/docs/IDB201_DSC_Reading_Plan.xlsx
@@ -680,7 +680,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• OPTIONAL sections are enrichment for honors students and feed Assignment 2 research topics.</t>
+          <t>• OPTIONAL sections are enrichment for honors students and feed group-project research topics.</t>
         </is>
       </c>
     </row>
@@ -1772,13 +1772,13 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Assignment 2</t>
+          <t>Group project</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr"/>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Good material for Assignment 2 research topics.</t>
+          <t>Good material for group-project research topics.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,11 @@
           <t>Học trên lớp</t>
         </is>
       </c>
-      <c r="J21" s="12" t="inlineStr"/>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>Duplicates and DISTINCT: bag semantics is guided self-study</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n">
@@ -3323,7 +3327,7 @@
       </c>
       <c r="J28" s="12" t="inlineStr">
         <is>
-          <t>Exercises used in Lab 5</t>
+          <t>Exercises used in Lab 1 (sessions 13–14)</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3703,7 @@
       </c>
       <c r="J37" s="12" t="inlineStr">
         <is>
-          <t>Python section (session 18); JDBC/ODBC self-study</t>
+          <t>Concepts and parameterized queries (session 18); Python access is optional self-study</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4247,7 @@
       </c>
       <c r="J50" s="12" t="inlineStr">
         <is>
-          <t>Specialization/generalization; practised in Lab 2</t>
+          <t>Specialization/generalization; practised in Lab 3</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4871,7 @@
       </c>
       <c r="J65" s="12" t="inlineStr">
         <is>
-          <t>Exercises used in Lab 7</t>
+          <t>Exercises used in the guided exercises of session 32</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6839,7 @@
       </c>
       <c r="J113" s="12" t="inlineStr">
         <is>
-          <t>Composite indexes (Lab 7)</t>
+          <t>Composite indexes (Lab 4)</t>
         </is>
       </c>
     </row>
@@ -9523,7 +9527,7 @@
       </c>
       <c r="J178" s="12" t="inlineStr">
         <is>
-          <t>Useful background for the Lab 8 experiments</t>
+          <t>Useful background for the Lab 4 experiments</t>
         </is>
       </c>
     </row>
@@ -9567,7 +9571,7 @@
       </c>
       <c r="J179" s="12" t="inlineStr">
         <is>
-          <t>How to design fair experiments (Assignment 2)</t>
+          <t>How to design fair experiments (group project)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild the DSC reading plan for the T-SQL chapter and trimmed internals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsfsusx3YZQC9pVr8xoQKL
</commit_message>
<xml_diff>
--- a/docs/IDB201_DSC_Reading_Plan.xlsx
+++ b/docs/IDB201_DSC_Reading_Plan.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +75,11 @@
         <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,13 +128,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -497,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -581,13 +589,13 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.211864406779661</v>
+        <v>0.2141756548536209</v>
       </c>
     </row>
     <row r="7">
@@ -602,13 +610,13 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>0.1078582434514638</v>
+        <v>0.1055469953775039</v>
       </c>
     </row>
     <row r="8">
@@ -666,33 +674,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>• IN CLASS pages average about 14 pages per theory session; students read them before class (flipped preparation).</t>
+          <t>• IN CLASS pages average about 11 pages per theory session (see 'Session load'); students read them before class (flipped preparation). C8 is the heaviest at about 18 pages per session because §14.3 (B+-trees) is read in full.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• SELF-STUDY is required and is checked through labs, progress tests and the final exam.</t>
+          <t>• Since 2026-10-14, §5.2–5.3 (functions, procedures, triggers) are taught in the T-SQL chapter C5, together with the Microsoft T-SQL reference.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• OPTIONAL sections are enrichment for honors students and feed group-project research topics.</t>
+          <t>• SELF-STUDY is required and is checked through labs, progress tests and the final exam.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>• LATER marks material that belongs to later BCS_AD courses (DSI201, DAM311, DPY391, BDI302c, MLD301).</t>
+          <t>• OPTIONAL sections are enrichment for honors students and feed group-project research topics.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>• LATER marks material that belongs to later BCS_AD courses (DSI201, DAM311, DPY391, BDI302c, MLD301).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>• Online chapters 27–32 have no page numbers in the printed table of contents.</t>
         </is>
@@ -961,27 +976,27 @@
           <t>183–240</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>SELF-STUDY</t>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>IN CLASS</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C4, C5</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>17–18</t>
+          <t>17–25</t>
         </is>
       </c>
       <c r="H6" s="12" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>Only the parts that support the academic goals are taught; procedural SQL is optional.</t>
+          <t>§5.1 and §5.4 support the academic goals (C4); §5.2–5.3 are the basis of the T-SQL programming chapter C5 (CLO4), taught together with the T-SQL reference.</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1026,12 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C6</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>21–25</t>
+          <t>27–31</t>
         </is>
       </c>
       <c r="H7" s="12" t="n">
@@ -1054,12 +1069,12 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>26–32</t>
+          <t>32–38</t>
         </is>
       </c>
       <c r="H8" s="12" t="n">
@@ -1090,7 +1105,7 @@
           <t>365–402</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
@@ -1131,7 +1146,7 @@
           <t>403–466</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1172,7 +1187,7 @@
           <t>467–518</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1213,7 +1228,7 @@
           <t>519–558</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1254,19 +1269,19 @@
           <t>559–586</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>41</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr"/>
@@ -1302,12 +1317,12 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>35–36</t>
+          <t>41</t>
         </is>
       </c>
       <c r="H14" s="12" t="n">
@@ -1345,20 +1360,20 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>36–40</t>
+          <t>42–44, 48</t>
         </is>
       </c>
       <c r="H15" s="12" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>B+-trees and hashing: official description names indexing (CLO6).</t>
+          <t>B+-trees and hashing at the level of main ideas and I/O cost: official description names indexing (CLO6). Students have not yet taken CSD203.</t>
         </is>
       </c>
     </row>
@@ -1388,12 +1403,12 @@
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>41–43, 46</t>
+          <t>45–46, 48</t>
         </is>
       </c>
       <c r="H16" s="12" t="n">
@@ -1431,20 +1446,20 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>44–46</t>
+          <t>47–48</t>
         </is>
       </c>
       <c r="H17" s="12" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Equivalence rules, estimation and join ordering (CLO6); official description names query optimization.</t>
+          <t>Equivalence rules and reading execution plans (CLO6); official description names query optimization. Estimation is self-study and join ordering by dynamic programming is optional.</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1489,12 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>47–49, 53</t>
+          <t>49–51, 53</t>
         </is>
       </c>
       <c r="H18" s="12" t="n">
@@ -1517,12 +1532,12 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>50–53</t>
+          <t>51–53</t>
         </is>
       </c>
       <c r="H19" s="12" t="n">
@@ -1530,7 +1545,7 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>Two-phase locking, deadlocks, snapshot isolation (CLO7). Other protocols are self-study.</t>
+          <t>Two-phase locking (main idea, lock point), deadlocks, phantoms; snapshot isolation as an overview (CLO7). Other protocols are self-study.</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1568,7 @@
           <t>907–960</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
@@ -1596,7 +1611,7 @@
           <t>961–1002</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1637,7 +1652,7 @@
           <t>1003–1038</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1678,7 +1693,7 @@
           <t>1039–1097</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1719,7 +1734,7 @@
           <t>1098–1174</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1760,14 +1775,14 @@
           <t>1175–1209</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -1801,7 +1816,7 @@
           <t>1210–1251</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1842,7 +1857,7 @@
           <t>1252–1286</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -1885,7 +1900,7 @@
           <t>1287–1298</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
@@ -1926,7 +1941,7 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
@@ -1967,14 +1982,14 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -2008,7 +2023,7 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -2045,7 +2060,7 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E32" s="16" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -2082,7 +2097,7 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
@@ -2123,7 +2138,7 @@
           <t>online</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E34" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
@@ -2535,12 +2550,12 @@
       <c r="G9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -2579,12 +2594,12 @@
       <c r="G10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -2623,12 +2638,12 @@
       <c r="G11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -2907,12 +2922,12 @@
       <c r="G18" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I18" s="14" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -3315,12 +3330,12 @@
       <c r="G28" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I28" s="14" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -3607,12 +3622,12 @@
       <c r="G35" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H35" s="14" t="inlineStr">
+      <c r="H35" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I35" s="14" t="inlineStr">
+      <c r="I35" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -3651,12 +3666,12 @@
       <c r="G36" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="H36" s="14" t="inlineStr">
+      <c r="H36" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I36" s="14" t="inlineStr">
+      <c r="I36" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -3735,19 +3750,19 @@
       <c r="G38" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H38" s="15" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="I38" s="15" t="inlineStr">
-        <is>
-          <t>Đọc thêm / đề tài nghiên cứu</t>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>IN CLASS</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>Học trên lớp</t>
         </is>
       </c>
       <c r="J38" s="12" t="inlineStr">
         <is>
-          <t>Optional Appendix A; useful for the project</t>
+          <t>T-SQL functions and stored procedures (sessions 20–21); loops over query results and T-SQL cursors (session 23); Lab 3</t>
         </is>
       </c>
     </row>
@@ -3779,19 +3794,19 @@
       <c r="G39" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H39" s="15" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="I39" s="15" t="inlineStr">
-        <is>
-          <t>Đọc thêm / đề tài nghiên cứu</t>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>IN CLASS</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>Học trên lớp</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
         <is>
-          <t>Optional Appendix A</t>
+          <t>AFTER and INSTEAD OF triggers, when not to use triggers (session 22); Lab 3</t>
         </is>
       </c>
     </row>
@@ -3867,12 +3882,12 @@
       <c r="G41" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H41" s="14" t="inlineStr">
+      <c r="H41" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I41" s="14" t="inlineStr">
+      <c r="I41" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -3911,12 +3926,12 @@
       <c r="G42" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="H42" s="14" t="inlineStr">
+      <c r="H42" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I42" s="14" t="inlineStr">
+      <c r="I42" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -4203,7 +4218,7 @@
       </c>
       <c r="J49" s="12" t="inlineStr">
         <is>
-          <t>Session 23</t>
+          <t>Session 29</t>
         </is>
       </c>
     </row>
@@ -4235,19 +4250,19 @@
       <c r="G50" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H50" s="14" t="inlineStr">
+      <c r="H50" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I50" s="14" t="inlineStr">
+      <c r="I50" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J50" s="12" t="inlineStr">
         <is>
-          <t>Specialization/generalization; practised in Lab 3</t>
+          <t>Specialization/generalization; practised in Lab 4</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4334,12 @@
       <c r="G52" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H52" s="14" t="inlineStr">
+      <c r="H52" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I52" s="14" t="inlineStr">
+      <c r="I52" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -4363,12 +4378,12 @@
       <c r="G53" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="14" t="inlineStr">
+      <c r="H53" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I53" s="14" t="inlineStr">
+      <c r="I53" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -4403,12 +4418,12 @@
       <c r="G54" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H54" s="14" t="inlineStr">
+      <c r="H54" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I54" s="14" t="inlineStr">
+      <c r="I54" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -4663,7 +4678,7 @@
       </c>
       <c r="J60" s="12" t="inlineStr">
         <is>
-          <t>MVDs and 4NF, overview (session 31)</t>
+          <t>MVDs and 4NF, overview (session 37)</t>
         </is>
       </c>
     </row>
@@ -4695,12 +4710,12 @@
       <c r="G61" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H61" s="15" t="inlineStr">
+      <c r="H61" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I61" s="15" t="inlineStr">
+      <c r="I61" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -4779,12 +4794,12 @@
       <c r="G63" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H63" s="14" t="inlineStr">
+      <c r="H63" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I63" s="14" t="inlineStr">
+      <c r="I63" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -4819,12 +4834,12 @@
       <c r="G64" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H64" s="15" t="inlineStr">
+      <c r="H64" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I64" s="15" t="inlineStr">
+      <c r="I64" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -4859,19 +4874,19 @@
       <c r="G65" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="H65" s="14" t="inlineStr">
+      <c r="H65" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I65" s="14" t="inlineStr">
+      <c r="I65" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
         <is>
-          <t>Exercises used in the guided exercises of session 32</t>
+          <t>Exercises used in the guided exercises of session 38</t>
         </is>
       </c>
     </row>
@@ -4903,12 +4918,12 @@
       <c r="G66" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H66" s="15" t="inlineStr">
+      <c r="H66" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I66" s="15" t="inlineStr">
+      <c r="I66" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -4947,12 +4962,12 @@
       <c r="G67" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H67" s="16" t="inlineStr">
+      <c r="H67" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I67" s="16" t="inlineStr">
+      <c r="I67" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -4987,12 +5002,12 @@
       <c r="G68" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H68" s="16" t="inlineStr">
+      <c r="H68" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I68" s="16" t="inlineStr">
+      <c r="I68" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5031,12 +5046,12 @@
       <c r="G69" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H69" s="16" t="inlineStr">
+      <c r="H69" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I69" s="16" t="inlineStr">
+      <c r="I69" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5071,12 +5086,12 @@
       <c r="G70" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="H70" s="16" t="inlineStr">
+      <c r="H70" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I70" s="16" t="inlineStr">
+      <c r="I70" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5111,12 +5126,12 @@
       <c r="G71" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H71" s="16" t="inlineStr">
+      <c r="H71" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I71" s="16" t="inlineStr">
+      <c r="I71" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5151,12 +5166,12 @@
       <c r="G72" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H72" s="16" t="inlineStr">
+      <c r="H72" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I72" s="16" t="inlineStr">
+      <c r="I72" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5191,12 +5206,12 @@
       <c r="G73" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H73" s="16" t="inlineStr">
+      <c r="H73" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I73" s="16" t="inlineStr">
+      <c r="I73" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5231,12 +5246,12 @@
       <c r="G74" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H74" s="16" t="inlineStr">
+      <c r="H74" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I74" s="16" t="inlineStr">
+      <c r="I74" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5271,12 +5286,12 @@
       <c r="G75" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H75" s="16" t="inlineStr">
+      <c r="H75" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I75" s="16" t="inlineStr">
+      <c r="I75" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5311,12 +5326,12 @@
       <c r="G76" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H76" s="16" t="inlineStr">
+      <c r="H76" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I76" s="16" t="inlineStr">
+      <c r="I76" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5351,12 +5366,12 @@
       <c r="G77" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H77" s="16" t="inlineStr">
+      <c r="H77" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I77" s="16" t="inlineStr">
+      <c r="I77" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5391,12 +5406,12 @@
       <c r="G78" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="H78" s="14" t="inlineStr">
+      <c r="H78" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I78" s="14" t="inlineStr">
+      <c r="I78" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -5435,12 +5450,12 @@
       <c r="G79" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H79" s="16" t="inlineStr">
+      <c r="H79" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I79" s="16" t="inlineStr">
+      <c r="I79" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5479,12 +5494,12 @@
       <c r="G80" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="H80" s="16" t="inlineStr">
+      <c r="H80" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I80" s="16" t="inlineStr">
+      <c r="I80" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5519,12 +5534,12 @@
       <c r="G81" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H81" s="15" t="inlineStr">
+      <c r="H81" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I81" s="15" t="inlineStr">
+      <c r="I81" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -5563,12 +5578,12 @@
       <c r="G82" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H82" s="16" t="inlineStr">
+      <c r="H82" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I82" s="16" t="inlineStr">
+      <c r="I82" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5603,12 +5618,12 @@
       <c r="G83" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H83" s="16" t="inlineStr">
+      <c r="H83" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I83" s="16" t="inlineStr">
+      <c r="I83" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5643,12 +5658,12 @@
       <c r="G84" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H84" s="15" t="inlineStr">
+      <c r="H84" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I84" s="15" t="inlineStr">
+      <c r="I84" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -5687,12 +5702,12 @@
       <c r="G85" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H85" s="16" t="inlineStr">
+      <c r="H85" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I85" s="16" t="inlineStr">
+      <c r="I85" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5727,12 +5742,12 @@
       <c r="G86" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H86" s="16" t="inlineStr">
+      <c r="H86" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I86" s="16" t="inlineStr">
+      <c r="I86" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5767,12 +5782,12 @@
       <c r="G87" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H87" s="16" t="inlineStr">
+      <c r="H87" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I87" s="16" t="inlineStr">
+      <c r="I87" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5807,12 +5822,12 @@
       <c r="G88" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H88" s="16" t="inlineStr">
+      <c r="H88" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I88" s="16" t="inlineStr">
+      <c r="I88" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5847,12 +5862,12 @@
       <c r="G89" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H89" s="15" t="inlineStr">
+      <c r="H89" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I89" s="15" t="inlineStr">
+      <c r="I89" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -5891,12 +5906,12 @@
       <c r="G90" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="H90" s="16" t="inlineStr">
+      <c r="H90" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I90" s="16" t="inlineStr">
+      <c r="I90" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5931,12 +5946,12 @@
       <c r="G91" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="H91" s="16" t="inlineStr">
+      <c r="H91" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I91" s="16" t="inlineStr">
+      <c r="I91" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -5975,12 +5990,12 @@
       <c r="G92" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="H92" s="16" t="inlineStr">
+      <c r="H92" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I92" s="16" t="inlineStr">
+      <c r="I92" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -6015,12 +6030,12 @@
       <c r="G93" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H93" s="14" t="inlineStr">
+      <c r="H93" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I93" s="14" t="inlineStr">
+      <c r="I93" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -6059,12 +6074,12 @@
       <c r="G94" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H94" s="16" t="inlineStr">
+      <c r="H94" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I94" s="16" t="inlineStr">
+      <c r="I94" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -6099,12 +6114,12 @@
       <c r="G95" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H95" s="15" t="inlineStr">
+      <c r="H95" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I95" s="15" t="inlineStr">
+      <c r="I95" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6139,12 +6154,12 @@
       <c r="G96" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H96" s="15" t="inlineStr">
+      <c r="H96" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I96" s="15" t="inlineStr">
+      <c r="I96" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6179,12 +6194,12 @@
       <c r="G97" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H97" s="16" t="inlineStr">
+      <c r="H97" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I97" s="16" t="inlineStr">
+      <c r="I97" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -6219,12 +6234,12 @@
       <c r="G98" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H98" s="14" t="inlineStr">
+      <c r="H98" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I98" s="14" t="inlineStr">
+      <c r="I98" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -6263,12 +6278,12 @@
       <c r="G99" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H99" s="16" t="inlineStr">
+      <c r="H99" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I99" s="16" t="inlineStr">
+      <c r="I99" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -6423,12 +6438,12 @@
       <c r="G103" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H103" s="14" t="inlineStr">
+      <c r="H103" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I103" s="14" t="inlineStr">
+      <c r="I103" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -6503,12 +6518,12 @@
       <c r="G105" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H105" s="15" t="inlineStr">
+      <c r="H105" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I105" s="15" t="inlineStr">
+      <c r="I105" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6547,12 +6562,12 @@
       <c r="G106" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H106" s="15" t="inlineStr">
+      <c r="H106" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I106" s="15" t="inlineStr">
+      <c r="I106" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6587,12 +6602,12 @@
       <c r="G107" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H107" s="14" t="inlineStr">
+      <c r="H107" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I107" s="14" t="inlineStr">
+      <c r="I107" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -6717,7 +6732,11 @@
           <t>Học trên lớp</t>
         </is>
       </c>
-      <c r="J110" s="12" t="inlineStr"/>
+      <c r="J110" s="12" t="inlineStr">
+        <is>
+          <t>Structure, search and height (session 42); insertion, deletion main idea (session 43)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="n">
@@ -6747,12 +6766,12 @@
       <c r="G111" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="H111" s="14" t="inlineStr">
+      <c r="H111" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I111" s="14" t="inlineStr">
+      <c r="I111" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -6797,7 +6816,11 @@
           <t>Học trên lớp</t>
         </is>
       </c>
-      <c r="J112" s="12" t="inlineStr"/>
+      <c r="J112" s="12" t="inlineStr">
+        <is>
+          <t>Session 43</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="12" t="n">
@@ -6827,19 +6850,19 @@
       <c r="G113" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H113" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I113" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H113" s="16" t="inlineStr">
+        <is>
+          <t>SELF-STUDY</t>
+        </is>
+      </c>
+      <c r="I113" s="16" t="inlineStr">
+        <is>
+          <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
       </c>
       <c r="J113" s="12" t="inlineStr">
         <is>
-          <t>Composite indexes (Lab 4)</t>
+          <t>Composite indexes; used in Lab 5 (part 1)</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6904,11 @@
           <t>Học trên lớp</t>
         </is>
       </c>
-      <c r="J114" s="12" t="inlineStr"/>
+      <c r="J114" s="12" t="inlineStr">
+        <is>
+          <t>Session 43</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="n">
@@ -6911,12 +6938,12 @@
       <c r="G115" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H115" s="15" t="inlineStr">
+      <c r="H115" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I115" s="15" t="inlineStr">
+      <c r="I115" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6955,12 +6982,12 @@
       <c r="G116" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H116" s="15" t="inlineStr">
+      <c r="H116" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I116" s="15" t="inlineStr">
+      <c r="I116" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -6995,12 +7022,12 @@
       <c r="G117" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H117" s="16" t="inlineStr">
+      <c r="H117" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I117" s="16" t="inlineStr">
+      <c r="I117" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -7035,12 +7062,12 @@
       <c r="G118" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H118" s="14" t="inlineStr">
+      <c r="H118" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I118" s="14" t="inlineStr">
+      <c r="I118" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7207,7 +7234,7 @@
       </c>
       <c r="J122" s="12" t="inlineStr">
         <is>
-          <t>External merge sort</t>
+          <t>External merge sort, main idea (session 45)</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7278,7 @@
       </c>
       <c r="J123" s="12" t="inlineStr">
         <is>
-          <t>Nested-loop, merge and hash joins</t>
+          <t>Nested-loop, merge and hash joins; cost comparison (session 46)</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7310,12 @@
       <c r="G124" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H124" s="14" t="inlineStr">
+      <c r="H124" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I124" s="14" t="inlineStr">
+      <c r="I124" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7323,12 +7350,12 @@
       <c r="G125" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H125" s="14" t="inlineStr">
+      <c r="H125" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I125" s="14" t="inlineStr">
+      <c r="I125" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7367,12 +7394,12 @@
       <c r="G126" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H126" s="15" t="inlineStr">
+      <c r="H126" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I126" s="15" t="inlineStr">
+      <c r="I126" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -7407,12 +7434,12 @@
       <c r="G127" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="H127" s="14" t="inlineStr">
+      <c r="H127" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I127" s="14" t="inlineStr">
+      <c r="I127" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7531,12 +7558,12 @@
       <c r="G130" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="H130" s="14" t="inlineStr">
+      <c r="H130" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I130" s="14" t="inlineStr">
+      <c r="I130" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7575,19 +7602,19 @@
       <c r="G131" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H131" s="13" t="inlineStr">
-        <is>
-          <t>IN CLASS</t>
-        </is>
-      </c>
-      <c r="I131" s="13" t="inlineStr">
-        <is>
-          <t>Học trên lớp</t>
+      <c r="H131" s="14" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="I131" s="14" t="inlineStr">
+        <is>
+          <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
         <is>
-          <t>Dynamic programming for join order</t>
+          <t>Dynamic programming for join order; optional self-study, needs CSD203 (S2)</t>
         </is>
       </c>
     </row>
@@ -7619,19 +7646,19 @@
       <c r="G132" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H132" s="15" t="inlineStr">
+      <c r="H132" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I132" s="15" t="inlineStr">
+      <c r="I132" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
       </c>
       <c r="J132" s="12" t="inlineStr">
         <is>
-          <t>Links to views (Ch. 7 of the course)</t>
+          <t>Links to views (C4, session 15)</t>
         </is>
       </c>
     </row>
@@ -7663,12 +7690,12 @@
       <c r="G133" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H133" s="16" t="inlineStr">
+      <c r="H133" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I133" s="16" t="inlineStr">
+      <c r="I133" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -7703,12 +7730,12 @@
       <c r="G134" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H134" s="14" t="inlineStr">
+      <c r="H134" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I134" s="14" t="inlineStr">
+      <c r="I134" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -7823,12 +7850,12 @@
       <c r="G137" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H137" s="14" t="inlineStr">
+      <c r="H137" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I137" s="14" t="inlineStr">
+      <c r="I137" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8121,7 +8148,11 @@
           <t>Học trên lớp</t>
         </is>
       </c>
-      <c r="J144" s="12" t="inlineStr"/>
+      <c r="J144" s="12" t="inlineStr">
+        <is>
+          <t>Session 49, with BEGIN TRAN / COMMIT / ROLLBACK in T-SQL</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="n">
@@ -8151,12 +8182,12 @@
       <c r="G145" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H145" s="14" t="inlineStr">
+      <c r="H145" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I145" s="14" t="inlineStr">
+      <c r="I145" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8203,7 +8234,7 @@
       </c>
       <c r="J146" s="12" t="inlineStr">
         <is>
-          <t>2PL and its correctness</t>
+          <t>2PL main idea and the lock point (session 51)</t>
         </is>
       </c>
     </row>
@@ -8275,12 +8306,12 @@
       <c r="G148" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H148" s="14" t="inlineStr">
+      <c r="H148" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I148" s="14" t="inlineStr">
+      <c r="I148" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8359,12 +8390,12 @@
       <c r="G150" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H150" s="14" t="inlineStr">
+      <c r="H150" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I150" s="14" t="inlineStr">
+      <c r="I150" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8399,12 +8430,12 @@
       <c r="G151" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H151" s="15" t="inlineStr">
+      <c r="H151" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I151" s="15" t="inlineStr">
+      <c r="I151" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -8439,12 +8470,12 @@
       <c r="G152" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H152" s="14" t="inlineStr">
+      <c r="H152" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I152" s="14" t="inlineStr">
+      <c r="I152" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8495,7 +8526,7 @@
       </c>
       <c r="J153" s="12" t="inlineStr">
         <is>
-          <t>Write skew</t>
+          <t>Overview, write skew (session 52)</t>
         </is>
       </c>
     </row>
@@ -8527,12 +8558,12 @@
       <c r="G154" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H154" s="14" t="inlineStr">
+      <c r="H154" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I154" s="14" t="inlineStr">
+      <c r="I154" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8567,12 +8598,12 @@
       <c r="G155" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="H155" s="16" t="inlineStr">
+      <c r="H155" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I155" s="16" t="inlineStr">
+      <c r="I155" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -8607,12 +8638,12 @@
       <c r="G156" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="H156" s="14" t="inlineStr">
+      <c r="H156" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I156" s="14" t="inlineStr">
+      <c r="I156" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8687,12 +8718,12 @@
       <c r="G158" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H158" s="14" t="inlineStr">
+      <c r="H158" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I158" s="14" t="inlineStr">
+      <c r="I158" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8771,12 +8802,12 @@
       <c r="G160" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H160" s="14" t="inlineStr">
+      <c r="H160" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I160" s="14" t="inlineStr">
+      <c r="I160" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8815,12 +8846,12 @@
       <c r="G161" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H161" s="14" t="inlineStr">
+      <c r="H161" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I161" s="14" t="inlineStr">
+      <c r="I161" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8855,12 +8886,12 @@
       <c r="G162" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H162" s="14" t="inlineStr">
+      <c r="H162" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I162" s="14" t="inlineStr">
+      <c r="I162" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -8895,12 +8926,12 @@
       <c r="G163" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H163" s="16" t="inlineStr">
+      <c r="H163" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I163" s="16" t="inlineStr">
+      <c r="I163" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -8935,12 +8966,12 @@
       <c r="G164" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H164" s="16" t="inlineStr">
+      <c r="H164" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I164" s="16" t="inlineStr">
+      <c r="I164" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -8975,19 +9006,19 @@
       <c r="G165" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H165" s="15" t="inlineStr">
+      <c r="H165" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I165" s="15" t="inlineStr">
+      <c r="I165" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
       </c>
       <c r="J165" s="12" t="inlineStr">
         <is>
-          <t>Research Corner reading for strong students</t>
+          <t>Optional reading for strong students</t>
         </is>
       </c>
     </row>
@@ -9019,12 +9050,12 @@
       <c r="G166" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H166" s="16" t="inlineStr">
+      <c r="H166" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I166" s="16" t="inlineStr">
+      <c r="I166" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9059,12 +9090,12 @@
       <c r="G167" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="H167" s="14" t="inlineStr">
+      <c r="H167" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I167" s="14" t="inlineStr">
+      <c r="I167" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -9099,12 +9130,12 @@
       <c r="G168" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="H168" s="16" t="inlineStr">
+      <c r="H168" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I168" s="16" t="inlineStr">
+      <c r="I168" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9143,12 +9174,12 @@
       <c r="G169" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="H169" s="16" t="inlineStr">
+      <c r="H169" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I169" s="16" t="inlineStr">
+      <c r="I169" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9183,12 +9214,12 @@
       <c r="G170" s="12" t="n">
         <v>59</v>
       </c>
-      <c r="H170" s="16" t="inlineStr">
+      <c r="H170" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I170" s="16" t="inlineStr">
+      <c r="I170" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9223,12 +9254,12 @@
       <c r="G171" s="12" t="n">
         <v>77</v>
       </c>
-      <c r="H171" s="16" t="inlineStr">
+      <c r="H171" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I171" s="16" t="inlineStr">
+      <c r="I171" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9263,12 +9294,12 @@
       <c r="G172" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H172" s="15" t="inlineStr">
+      <c r="H172" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I172" s="15" t="inlineStr">
+      <c r="I172" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9307,12 +9338,12 @@
       <c r="G173" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H173" s="15" t="inlineStr">
+      <c r="H173" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I173" s="15" t="inlineStr">
+      <c r="I173" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9351,12 +9382,12 @@
       <c r="G174" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H174" s="15" t="inlineStr">
+      <c r="H174" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I174" s="15" t="inlineStr">
+      <c r="I174" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9391,12 +9422,12 @@
       <c r="G175" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H175" s="16" t="inlineStr">
+      <c r="H175" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I175" s="16" t="inlineStr">
+      <c r="I175" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9431,12 +9462,12 @@
       <c r="G176" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="H176" s="15" t="inlineStr">
+      <c r="H176" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I176" s="15" t="inlineStr">
+      <c r="I176" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9475,12 +9506,12 @@
       <c r="G177" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="H177" s="15" t="inlineStr">
+      <c r="H177" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I177" s="15" t="inlineStr">
+      <c r="I177" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9515,19 +9546,19 @@
       <c r="G178" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="H178" s="15" t="inlineStr">
+      <c r="H178" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I178" s="15" t="inlineStr">
+      <c r="I178" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
       </c>
       <c r="J178" s="12" t="inlineStr">
         <is>
-          <t>Useful background for the Lab 4 experiments</t>
+          <t>Useful background for the Lab 5 experiments</t>
         </is>
       </c>
     </row>
@@ -9559,12 +9590,12 @@
       <c r="G179" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H179" s="15" t="inlineStr">
+      <c r="H179" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I179" s="15" t="inlineStr">
+      <c r="I179" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9603,12 +9634,12 @@
       <c r="G180" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="H180" s="16" t="inlineStr">
+      <c r="H180" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I180" s="16" t="inlineStr">
+      <c r="I180" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9643,12 +9674,12 @@
       <c r="G181" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="H181" s="16" t="inlineStr">
+      <c r="H181" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I181" s="16" t="inlineStr">
+      <c r="I181" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9685,12 +9716,12 @@
       <c r="G182" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H182" s="14" t="inlineStr">
+      <c r="H182" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I182" s="14" t="inlineStr">
+      <c r="I182" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -9723,12 +9754,12 @@
       <c r="E183" s="12" t="n"/>
       <c r="F183" s="12" t="n"/>
       <c r="G183" s="12" t="n"/>
-      <c r="H183" s="14" t="inlineStr">
+      <c r="H183" s="16" t="inlineStr">
         <is>
           <t>SELF-STUDY</t>
         </is>
       </c>
-      <c r="I183" s="14" t="inlineStr">
+      <c r="I183" s="16" t="inlineStr">
         <is>
           <t>Tự học có hướng dẫn (bắt buộc)</t>
         </is>
@@ -9761,12 +9792,12 @@
       <c r="E184" s="12" t="n"/>
       <c r="F184" s="12" t="n"/>
       <c r="G184" s="12" t="n"/>
-      <c r="H184" s="15" t="inlineStr">
+      <c r="H184" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I184" s="15" t="inlineStr">
+      <c r="I184" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -9795,12 +9826,12 @@
       <c r="E185" s="12" t="n"/>
       <c r="F185" s="12" t="n"/>
       <c r="G185" s="12" t="n"/>
-      <c r="H185" s="16" t="inlineStr">
+      <c r="H185" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I185" s="16" t="inlineStr">
+      <c r="I185" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9829,12 +9860,12 @@
       <c r="E186" s="12" t="n"/>
       <c r="F186" s="12" t="n"/>
       <c r="G186" s="12" t="n"/>
-      <c r="H186" s="16" t="inlineStr">
+      <c r="H186" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I186" s="16" t="inlineStr">
+      <c r="I186" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9863,12 +9894,12 @@
       <c r="E187" s="12" t="n"/>
       <c r="F187" s="12" t="n"/>
       <c r="G187" s="12" t="n"/>
-      <c r="H187" s="16" t="inlineStr">
+      <c r="H187" s="15" t="inlineStr">
         <is>
           <t>LATER</t>
         </is>
       </c>
-      <c r="I187" s="16" t="inlineStr">
+      <c r="I187" s="15" t="inlineStr">
         <is>
           <t>Ngoài phạm vi – học ở môn sau</t>
         </is>
@@ -9897,12 +9928,12 @@
       <c r="E188" s="12" t="n"/>
       <c r="F188" s="12" t="n"/>
       <c r="G188" s="12" t="n"/>
-      <c r="H188" s="15" t="inlineStr">
+      <c r="H188" s="14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="I188" s="15" t="inlineStr">
+      <c r="I188" s="14" t="inlineStr">
         <is>
           <t>Đọc thêm / đề tài nghiên cứu</t>
         </is>
@@ -10056,7 +10087,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Ch. 4, Ch. 5</t>
+          <t>Ch. 4, §5.1, §5.4</t>
         </is>
       </c>
       <c r="C5" s="12" t="n">
@@ -10079,24 +10110,24 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>C5 E-R model</t>
+          <t>C5 Programming the server in T-SQL</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Ch. 6</t>
+          <t>§5.2, §5.3</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>21–24 (4)</t>
+          <t>20–23 (4)</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>9</v>
+        <v>3.8</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
@@ -10107,24 +10138,24 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>C6 Relational database design</t>
+          <t>C6 E-R model</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Ch. 7</t>
+          <t>Ch. 6</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>26–31 (6)</t>
+          <t>27–30 (4)</t>
         </is>
       </c>
       <c r="E7" s="12" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
@@ -10135,24 +10166,24 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>C7 Storage and indexing</t>
+          <t>C7 Relational database design</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Ch. 12, Ch. 13, Ch. 14</t>
+          <t>Ch. 7</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>35–38 (4)</t>
+          <t>32–37 (6)</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>14</v>
+        <v>6.5</v>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
@@ -10163,52 +10194,52 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>C8 Query processing and optimization</t>
+          <t>C8 Storage and indexing</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Ch. 15, Ch. 16</t>
+          <t>Ch. 12, Ch. 13, Ch. 14</t>
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>41–45 (5)</t>
+          <t>41–43 (3)</t>
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>17.7</v>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Heavy</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>C9 Transactions and concurrency</t>
+          <t>C9 Query processing and optimization</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Ch. 17, Ch. 18</t>
+          <t>Ch. 15, Ch. 16</t>
         </is>
       </c>
       <c r="C10" s="12" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>47–52 (6)</t>
+          <t>45–47 (3)</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>9.699999999999999</v>
+        <v>14.7</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -10219,24 +10250,24 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>C10 Recovery (mainly self-study)</t>
+          <t>C10 Transactions, concurrency control and recovery</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Ch. 19</t>
+          <t>Ch. 17, Ch. 18, Ch. 19</t>
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>54 (1)</t>
+          <t>49–52, 54 (5)</t>
         </is>
       </c>
       <c r="E11" s="12" t="n">
-        <v>11</v>
+        <v>13.8</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>

</xml_diff>